<commit_message>
Add Bardak Kapak sheet with Powerplast updated price
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SWKZcbZgtYv9SeBCDKuQUk
</commit_message>
<xml_diff>
--- a/fiyat_karsilastirma.xlsx
+++ b/fiyat_karsilastirma.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Karşılaştırma" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bardak Kapak" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,13 +17,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0&quot; adet&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000&quot; €&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0.00&quot; TL&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; € toplam&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
+    <numFmt numFmtId="169" formatCode="0.0000&quot; USD / adet&quot;"/>
+    <numFmt numFmtId="170" formatCode="#,##0.00&quot; USD&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +40,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="5">
@@ -61,7 +69,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -83,11 +91,44 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -117,15 +158,70 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0092D050"/>
+          <bgColor rgb="0092D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FF0000"/>
+          <bgColor rgb="00FF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -587,7 +683,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n"/>
+      <c r="A5" s="13" t="n"/>
       <c r="B5" s="7" t="n">
         <v>22500</v>
       </c>
@@ -605,7 +701,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
+      <c r="A6" s="13" t="n"/>
       <c r="B6" s="8" t="n">
         <v>0.106</v>
       </c>
@@ -624,7 +720,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
+      <c r="A7" s="13" t="n"/>
       <c r="B7" s="9">
         <f>B6*$B$1</f>
         <v/>
@@ -646,7 +742,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
+      <c r="A8" s="14" t="n"/>
       <c r="B8" s="10">
         <f>B5*B6</f>
         <v/>
@@ -703,7 +799,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n"/>
+      <c r="A11" s="13" t="n"/>
       <c r="B11" s="7" t="n">
         <v>15000</v>
       </c>
@@ -721,7 +817,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n"/>
+      <c r="A12" s="13" t="n"/>
       <c r="B12" s="8" t="n">
         <v>0.168</v>
       </c>
@@ -740,7 +836,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n"/>
+      <c r="A13" s="13" t="n"/>
       <c r="B13" s="9">
         <f>B12*$B$1</f>
         <v/>
@@ -762,7 +858,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n"/>
+      <c r="A14" s="14" t="n"/>
       <c r="B14" s="10">
         <f>B11*B12</f>
         <v/>
@@ -819,7 +915,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n"/>
+      <c r="A17" s="13" t="n"/>
       <c r="B17" s="7" t="n">
         <v>18000</v>
       </c>
@@ -837,7 +933,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n"/>
+      <c r="A18" s="13" t="n"/>
       <c r="B18" s="8" t="n">
         <v>0.218</v>
       </c>
@@ -856,7 +952,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n"/>
+      <c r="A19" s="13" t="n"/>
       <c r="B19" s="9">
         <f>B18*$B$1</f>
         <v/>
@@ -878,7 +974,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n"/>
+      <c r="A20" s="14" t="n"/>
       <c r="B20" s="10">
         <f>B17*B18</f>
         <v/>
@@ -989,4 +1085,324 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>24.06.2026 – Soğuk Bardak / Kapak Teklif Karşılaştırması</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Kur USD/TL</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>(görseldeki TL tutarlarından türetildi)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Powerplast bardak: USD / 1000 adet</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>← değiştirilebilir giriş</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Malzeme</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Miktar</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>POWERPLAST
+(eski: Packsel)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>S.N.A</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>SACEM</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>SHADKAR COMPANY</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>SOĞUK BARDAK</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C6" s="19">
+        <f>$B$3/1000</f>
+        <v/>
+      </c>
+      <c r="D6" s="19" t="n">
+        <v>0.0924</v>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>0.093</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>0.1065</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="20" t="n"/>
+      <c r="B7" s="20" t="n"/>
+      <c r="C7" s="21">
+        <f>$B6*C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="21">
+        <f>$B6*D6</f>
+        <v/>
+      </c>
+      <c r="E7" s="21">
+        <f>$B6*E6</f>
+        <v/>
+      </c>
+      <c r="F7" s="21">
+        <f>$B6*F6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="n"/>
+      <c r="B8" s="20" t="n"/>
+      <c r="C8" s="22">
+        <f>C7*$B$2</f>
+        <v/>
+      </c>
+      <c r="D8" s="22">
+        <f>D7*$B$2</f>
+        <v/>
+      </c>
+      <c r="E8" s="22">
+        <f>E7*$B$2</f>
+        <v/>
+      </c>
+      <c r="F8" s="22">
+        <f>F7*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>SOĞUK KAPAK</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>150000</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0.021</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>0.0285</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="n"/>
+      <c r="B10" s="20" t="n"/>
+      <c r="C10" s="21">
+        <f>$B9*C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="21">
+        <f>$B9*D9</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>$B9*E9</f>
+        <v/>
+      </c>
+      <c r="F10" s="21">
+        <f>$B9*F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="n"/>
+      <c r="B11" s="20" t="n"/>
+      <c r="C11" s="22">
+        <f>C10*$B$2</f>
+        <v/>
+      </c>
+      <c r="D11" s="22">
+        <f>D10*$B$2</f>
+        <v/>
+      </c>
+      <c r="E11" s="22">
+        <f>E10*$B$2</f>
+        <v/>
+      </c>
+      <c r="F11" s="22">
+        <f>F10*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>TOPLAM</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="25">
+        <f>C7+C10</f>
+        <v/>
+      </c>
+      <c r="D12" s="25">
+        <f>D7+D10</f>
+        <v/>
+      </c>
+      <c r="E12" s="25">
+        <f>E7+E10</f>
+        <v/>
+      </c>
+      <c r="F12" s="25">
+        <f>F7+F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="n"/>
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="26">
+        <f>C12*$B$2</f>
+        <v/>
+      </c>
+      <c r="D13" s="26">
+        <f>D12*$B$2</f>
+        <v/>
+      </c>
+      <c r="E13" s="26">
+        <f>E12*$B$2</f>
+        <v/>
+      </c>
+      <c r="F13" s="26">
+        <f>F12*$B$2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="62" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Ödeme</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="n"/>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>Powerplast: belirtilmedi (Packsel'de %30 peşin, kalan 30-60 gün vade idi)</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>%30 peşin, kalan 30-60-90 gün vade</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>%30 peşin, kalan ürün tesliminde</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="inlineStr">
+        <is>
+          <t>%50 peşin, kalan 60 gün vade</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Yeşil = en düşük, kırmızı = en yüksek. Powerplast bardak fiyatı B3'teki 63 USD/1000 adet varsayımıyla hesaplandı; kapak fiyatı Packsel teklifiyle aynı (0,032).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="C6:F6">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>C6=MIN($C6:$F6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>C6=MAX($C6:$F6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:F9">
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>C9=MIN($C9:$F9)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="2">
+      <formula>C9=MAX($C9:$F9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12:F12">
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>C12=MIN($C12:$F12)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>C12=MAX($C12:$F12)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>